<commit_message>
Adicionando algumas anotações no dicionário de dados - 14/04/2026
</commit_message>
<xml_diff>
--- a/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_de_dados_projeto.xlsx
+++ b/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_de_dados_projeto.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gusta\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B 789\Downloads\Projetos_ADSN_Einstein\Terceiro_Semestre\Projeto_Integrador\Documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D089A5-6B9D-4F66-8311-26DB66C06D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{469F5BF7-1942-432A-8289-DDFBF75692AC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16170" windowHeight="6060"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="87">
   <si>
     <t>Mnemônico</t>
   </si>
@@ -301,13 +300,16 @@
   <si>
     <t>Chave primaria de indetificação único da
 tabela "laboratorio"</t>
+  </si>
+  <si>
+    <t>pode ser char somente -&gt; (P, C e CT)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -719,24 +721,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -760,6 +744,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1094,73 +1096,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{064BA25E-541B-4771-AFA8-C0176CB4D374}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BT63"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.88671875" customWidth="1"/>
-    <col min="14" max="14" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.875" customWidth="1"/>
+    <col min="14" max="14" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.88671875" style="33"/>
-    <col min="26" max="26" width="20.33203125" style="33" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.25" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.875" style="33"/>
+    <col min="26" max="26" width="20.375" style="33" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="22" style="33" customWidth="1"/>
-    <col min="28" max="28" width="8.88671875" style="33"/>
-    <col min="29" max="29" width="14.44140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="30" max="32" width="8.88671875" style="33"/>
-    <col min="33" max="33" width="12.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.109375" style="33" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.88671875" style="33" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8.88671875" style="33"/>
-    <col min="38" max="38" width="19.109375" style="33" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="26.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.44140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="42" max="44" width="8.88671875" style="33"/>
-    <col min="45" max="45" width="12.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="22.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.88671875" style="33" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="18.88671875" style="33" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.88671875" style="33"/>
-    <col min="50" max="50" width="18.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="22.33203125" style="33" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="8.88671875" style="33"/>
-    <col min="53" max="53" width="14.44140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.44140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="55" max="56" width="8.88671875" style="33"/>
-    <col min="57" max="57" width="12.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="22.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.88671875" style="33" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="20.109375" style="33" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="8.88671875" style="33"/>
-    <col min="62" max="62" width="18.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="22.33203125" style="33" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="8.88671875" style="33"/>
-    <col min="65" max="65" width="14.44140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="66" max="68" width="8.88671875" style="33"/>
-    <col min="69" max="69" width="12.5546875" style="33" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.88671875" style="33" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="16.5546875" style="33" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.875" style="33"/>
+    <col min="29" max="29" width="14.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="30" max="32" width="8.875" style="33"/>
+    <col min="33" max="33" width="12.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.125" style="33" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.875" style="33"/>
+    <col min="38" max="38" width="19.125" style="33" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="26.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="14.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="42" max="44" width="8.875" style="33"/>
+    <col min="45" max="45" width="12.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="22.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="18.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="8.875" style="33"/>
+    <col min="50" max="50" width="18.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="22.375" style="33" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="8.875" style="33"/>
+    <col min="53" max="53" width="14.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="55" max="56" width="8.875" style="33"/>
+    <col min="57" max="57" width="12.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="22.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="20.125" style="33" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="8.875" style="33"/>
+    <col min="62" max="62" width="18.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="22.375" style="33" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="8.875" style="33"/>
+    <col min="65" max="65" width="14.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="66" max="68" width="8.875" style="33"/>
+    <col min="69" max="69" width="12.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="16.5" style="33" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" ht="18">
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -1172,21 +1174,21 @@
       <c r="J1" s="31"/>
       <c r="K1" s="31"/>
       <c r="L1" s="31"/>
-      <c r="N1" s="46" t="s">
+      <c r="N1" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="O1" s="47"/>
-      <c r="P1" s="47"/>
-      <c r="Q1" s="47"/>
-      <c r="R1" s="47"/>
-      <c r="S1" s="47"/>
-      <c r="T1" s="47"/>
-      <c r="U1" s="47"/>
-      <c r="V1" s="47"/>
-      <c r="W1" s="47"/>
-      <c r="X1" s="48"/>
-    </row>
-    <row r="2" spans="1:25" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="55"/>
+      <c r="V1" s="55"/>
+      <c r="W1" s="55"/>
+      <c r="X1" s="56"/>
+    </row>
+    <row r="2" spans="1:25" ht="31.5">
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
       <c r="D2" s="32"/>
@@ -1232,7 +1234,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" ht="28.5">
       <c r="B3" s="32"/>
       <c r="C3" s="32"/>
       <c r="D3" s="32"/>
@@ -1278,7 +1280,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" ht="18">
       <c r="B4" s="32"/>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -1324,7 +1326,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" ht="28.5">
       <c r="A5" s="27"/>
       <c r="B5" s="32"/>
       <c r="C5" s="32"/>
@@ -1367,11 +1369,11 @@
       <c r="W5" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="X5" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="X5" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" ht="28.5">
       <c r="A6" s="27"/>
       <c r="B6" s="32"/>
       <c r="C6" s="32"/>
@@ -1418,7 +1420,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" ht="18.75" thickBot="1">
       <c r="A7" s="27"/>
       <c r="B7" s="32"/>
       <c r="C7" s="32"/>
@@ -1465,7 +1467,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" ht="36" customHeight="1" thickBot="1">
       <c r="A8" s="27"/>
       <c r="B8" s="32"/>
       <c r="C8" s="32"/>
@@ -1479,7 +1481,7 @@
       <c r="K8" s="32"/>
       <c r="L8" s="32"/>
     </row>
-    <row r="9" spans="1:25" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:25" ht="22.9" customHeight="1" thickBot="1">
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
       <c r="D9" s="32"/>
@@ -1491,21 +1493,21 @@
       <c r="J9" s="32"/>
       <c r="K9" s="32"/>
       <c r="L9" s="32"/>
-      <c r="N9" s="49" t="s">
+      <c r="N9" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="O9" s="50"/>
-      <c r="P9" s="50"/>
-      <c r="Q9" s="50"/>
-      <c r="R9" s="50"/>
-      <c r="S9" s="50"/>
-      <c r="T9" s="50"/>
-      <c r="U9" s="50"/>
-      <c r="V9" s="50"/>
-      <c r="W9" s="50"/>
-      <c r="X9" s="51"/>
-    </row>
-    <row r="10" spans="1:25" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O9" s="58"/>
+      <c r="P9" s="58"/>
+      <c r="Q9" s="58"/>
+      <c r="R9" s="58"/>
+      <c r="S9" s="58"/>
+      <c r="T9" s="58"/>
+      <c r="U9" s="58"/>
+      <c r="V9" s="58"/>
+      <c r="W9" s="58"/>
+      <c r="X9" s="59"/>
+    </row>
+    <row r="10" spans="1:25" ht="32.25" thickBot="1">
       <c r="B10" s="32"/>
       <c r="C10" s="32"/>
       <c r="D10" s="32"/>
@@ -1551,7 +1553,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" ht="28.5">
       <c r="B11" s="32"/>
       <c r="C11" s="32"/>
       <c r="D11" s="32"/>
@@ -1597,7 +1599,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25">
       <c r="N12" s="8" t="s">
         <v>35</v>
       </c>
@@ -1632,7 +1634,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25">
       <c r="N13" s="8" t="s">
         <v>36</v>
       </c>
@@ -1667,7 +1669,10 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" ht="28.5">
+      <c r="L14" t="s">
+        <v>86</v>
+      </c>
       <c r="N14" s="26" t="s">
         <v>37</v>
       </c>
@@ -1702,7 +1707,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:25" ht="15" thickBot="1">
       <c r="B15" s="33"/>
       <c r="C15" s="33"/>
       <c r="D15" s="33"/>
@@ -1748,7 +1753,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" ht="36" customHeight="1">
       <c r="B16" s="33"/>
       <c r="C16" s="33"/>
       <c r="D16" s="33"/>
@@ -1774,7 +1779,7 @@
       <c r="X16" s="29"/>
       <c r="Y16" s="38"/>
     </row>
-    <row r="17" spans="2:26" ht="22.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:26" ht="22.9" customHeight="1" thickBot="1">
       <c r="B17" s="33"/>
       <c r="C17" s="33"/>
       <c r="D17" s="33"/>
@@ -1787,7 +1792,7 @@
       <c r="K17" s="33"/>
       <c r="L17" s="33"/>
     </row>
-    <row r="18" spans="2:26" ht="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:26" ht="18">
       <c r="B18" s="33"/>
       <c r="C18" s="33"/>
       <c r="D18" s="33"/>
@@ -1799,22 +1804,22 @@
       <c r="J18" s="33"/>
       <c r="K18" s="33"/>
       <c r="L18" s="33"/>
-      <c r="N18" s="46" t="s">
+      <c r="N18" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="O18" s="47"/>
-      <c r="P18" s="47"/>
-      <c r="Q18" s="47"/>
-      <c r="R18" s="47"/>
-      <c r="S18" s="47"/>
-      <c r="T18" s="47"/>
-      <c r="U18" s="47"/>
-      <c r="V18" s="47"/>
-      <c r="W18" s="47"/>
-      <c r="X18" s="48"/>
+      <c r="O18" s="55"/>
+      <c r="P18" s="55"/>
+      <c r="Q18" s="55"/>
+      <c r="R18" s="55"/>
+      <c r="S18" s="55"/>
+      <c r="T18" s="55"/>
+      <c r="U18" s="55"/>
+      <c r="V18" s="55"/>
+      <c r="W18" s="55"/>
+      <c r="X18" s="56"/>
       <c r="Z18" s="39"/>
     </row>
-    <row r="19" spans="2:26" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:26" ht="31.5">
       <c r="B19" s="33"/>
       <c r="C19" s="33"/>
       <c r="D19" s="33"/>
@@ -1860,7 +1865,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="2:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:26" ht="28.5">
       <c r="B20" s="33"/>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -1906,7 +1911,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:26">
       <c r="B21" s="33"/>
       <c r="C21" s="33"/>
       <c r="D21" s="33"/>
@@ -1952,7 +1957,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:26" ht="15" thickBot="1">
       <c r="B22" s="33"/>
       <c r="C22" s="33"/>
       <c r="D22" s="33"/>
@@ -1999,7 +2004,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="2:26" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:26" ht="42" customHeight="1">
       <c r="B23" s="33"/>
       <c r="C23" s="33"/>
       <c r="D23" s="33"/>
@@ -2012,7 +2017,7 @@
       <c r="K23" s="33"/>
       <c r="L23" s="33"/>
     </row>
-    <row r="24" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:26" ht="15" thickBot="1">
       <c r="B24" s="33"/>
       <c r="C24" s="33"/>
       <c r="D24" s="33"/>
@@ -2025,7 +2030,7 @@
       <c r="K24" s="33"/>
       <c r="L24" s="33"/>
     </row>
-    <row r="25" spans="2:26" ht="18" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:26" ht="18">
       <c r="B25" s="33"/>
       <c r="C25" s="33"/>
       <c r="D25" s="33"/>
@@ -2037,21 +2042,21 @@
       <c r="J25" s="33"/>
       <c r="K25" s="33"/>
       <c r="L25" s="33"/>
-      <c r="N25" s="46" t="s">
+      <c r="N25" s="54" t="s">
         <v>50</v>
       </c>
-      <c r="O25" s="47"/>
-      <c r="P25" s="47"/>
-      <c r="Q25" s="47"/>
-      <c r="R25" s="47"/>
-      <c r="S25" s="47"/>
-      <c r="T25" s="47"/>
-      <c r="U25" s="47"/>
-      <c r="V25" s="47"/>
-      <c r="W25" s="47"/>
-      <c r="X25" s="48"/>
-    </row>
-    <row r="26" spans="2:26" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O25" s="55"/>
+      <c r="P25" s="55"/>
+      <c r="Q25" s="55"/>
+      <c r="R25" s="55"/>
+      <c r="S25" s="55"/>
+      <c r="T25" s="55"/>
+      <c r="U25" s="55"/>
+      <c r="V25" s="55"/>
+      <c r="W25" s="55"/>
+      <c r="X25" s="56"/>
+    </row>
+    <row r="26" spans="2:26" ht="31.5">
       <c r="B26" s="33"/>
       <c r="C26" s="33"/>
       <c r="D26" s="33"/>
@@ -2097,7 +2102,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="2:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:26" ht="28.5">
       <c r="B27" s="33"/>
       <c r="C27" s="33"/>
       <c r="D27" s="33"/>
@@ -2143,7 +2148,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:26">
       <c r="B28" s="33"/>
       <c r="C28" s="33"/>
       <c r="D28" s="33"/>
@@ -2189,7 +2194,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:26">
       <c r="B29" s="33"/>
       <c r="C29" s="33"/>
       <c r="D29" s="33"/>
@@ -2235,7 +2240,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:26">
       <c r="B30" s="33"/>
       <c r="C30" s="33"/>
       <c r="D30" s="33"/>
@@ -2281,7 +2286,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="31" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:26" ht="15" thickBot="1">
       <c r="B31" s="33"/>
       <c r="C31" s="33"/>
       <c r="D31" s="33"/>
@@ -2327,7 +2332,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="32" spans="2:26" ht="41.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:26" ht="41.45" customHeight="1" thickBot="1">
       <c r="B32" s="33"/>
       <c r="C32" s="33"/>
       <c r="D32" s="33"/>
@@ -2340,7 +2345,7 @@
       <c r="K32" s="33"/>
       <c r="L32" s="33"/>
     </row>
-    <row r="33" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:24" ht="18">
       <c r="B33" s="33"/>
       <c r="C33" s="33"/>
       <c r="D33" s="33"/>
@@ -2352,21 +2357,21 @@
       <c r="J33" s="33"/>
       <c r="K33" s="33"/>
       <c r="L33" s="33"/>
-      <c r="N33" s="46" t="s">
+      <c r="N33" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="O33" s="47"/>
-      <c r="P33" s="47"/>
-      <c r="Q33" s="47"/>
-      <c r="R33" s="47"/>
-      <c r="S33" s="47"/>
-      <c r="T33" s="47"/>
-      <c r="U33" s="47"/>
-      <c r="V33" s="47"/>
-      <c r="W33" s="47"/>
-      <c r="X33" s="48"/>
-    </row>
-    <row r="34" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="O33" s="55"/>
+      <c r="P33" s="55"/>
+      <c r="Q33" s="55"/>
+      <c r="R33" s="55"/>
+      <c r="S33" s="55"/>
+      <c r="T33" s="55"/>
+      <c r="U33" s="55"/>
+      <c r="V33" s="55"/>
+      <c r="W33" s="55"/>
+      <c r="X33" s="56"/>
+    </row>
+    <row r="34" spans="2:24" ht="15">
       <c r="B34" s="33"/>
       <c r="C34" s="33"/>
       <c r="D34" s="33"/>
@@ -2378,41 +2383,41 @@
       <c r="J34" s="33"/>
       <c r="K34" s="33"/>
       <c r="L34" s="33"/>
-      <c r="N34" s="53" t="s">
+      <c r="N34" s="47" t="s">
         <v>65</v>
       </c>
-      <c r="O34" s="52" t="s">
+      <c r="O34" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="P34" s="52" t="s">
+      <c r="P34" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="Q34" s="52">
+      <c r="Q34" s="46">
         <v>10</v>
       </c>
-      <c r="R34" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S34" s="52" t="s">
+      <c r="R34" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S34" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="T34" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="U34" s="52" t="s">
+      <c r="T34" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="U34" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="V34" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="W34" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X34" s="56" t="s">
+      <c r="V34" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="W34" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X34" s="50" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="35" spans="2:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:24" ht="22.15" customHeight="1">
       <c r="B35" s="33"/>
       <c r="C35" s="33"/>
       <c r="D35" s="33"/>
@@ -2424,41 +2429,41 @@
       <c r="J35" s="33"/>
       <c r="K35" s="33"/>
       <c r="L35" s="33"/>
-      <c r="N35" s="53" t="s">
+      <c r="N35" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="O35" s="52" t="s">
+      <c r="O35" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="P35" s="52" t="s">
+      <c r="P35" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="Q35" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="R35" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S35" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="T35" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="U35" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="V35" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="W35" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X35" s="56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="Q35" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="R35" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S35" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="T35" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="U35" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="V35" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="W35" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X35" s="50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="2:24" ht="15">
       <c r="B36" s="33"/>
       <c r="C36" s="33"/>
       <c r="D36" s="33"/>
@@ -2470,41 +2475,41 @@
       <c r="J36" s="33"/>
       <c r="K36" s="33"/>
       <c r="L36" s="33"/>
-      <c r="N36" s="53" t="s">
+      <c r="N36" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="O36" s="52" t="s">
+      <c r="O36" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="P36" s="52" t="s">
+      <c r="P36" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="Q36" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="R36" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S36" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="T36" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="U36" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="V36" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="W36" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X36" s="56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="Q36" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="R36" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S36" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="T36" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="U36" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="V36" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="W36" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X36" s="50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="2:24" ht="15">
       <c r="B37" s="33"/>
       <c r="C37" s="33"/>
       <c r="D37" s="33"/>
@@ -2516,41 +2521,41 @@
       <c r="J37" s="33"/>
       <c r="K37" s="33"/>
       <c r="L37" s="33"/>
-      <c r="N37" s="53" t="s">
+      <c r="N37" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="O37" s="52" t="s">
+      <c r="O37" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="P37" s="52" t="s">
+      <c r="P37" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="Q37" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="R37" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S37" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="T37" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="U37" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="V37" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="W37" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X37" s="56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="Q37" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="R37" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S37" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="T37" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="U37" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="V37" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="W37" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X37" s="50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="2:24" ht="15">
       <c r="B38" s="33"/>
       <c r="C38" s="33"/>
       <c r="D38" s="33"/>
@@ -2562,41 +2567,41 @@
       <c r="J38" s="33"/>
       <c r="K38" s="33"/>
       <c r="L38" s="33"/>
-      <c r="N38" s="53" t="s">
+      <c r="N38" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="O38" s="52" t="s">
+      <c r="O38" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="P38" s="52" t="s">
+      <c r="P38" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="Q38" s="52">
+      <c r="Q38" s="46">
         <v>30</v>
       </c>
-      <c r="R38" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S38" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="T38" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="U38" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="V38" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="W38" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X38" s="56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="39" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="R38" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S38" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="T38" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="U38" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="V38" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="W38" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X38" s="50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="2:24" ht="15">
       <c r="B39" s="33"/>
       <c r="C39" s="33"/>
       <c r="D39" s="33"/>
@@ -2608,41 +2613,41 @@
       <c r="J39" s="33"/>
       <c r="K39" s="33"/>
       <c r="L39" s="33"/>
-      <c r="N39" s="53" t="s">
+      <c r="N39" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="O39" s="52" t="s">
+      <c r="O39" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="P39" s="52" t="s">
+      <c r="P39" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="Q39" s="52">
+      <c r="Q39" s="46">
         <v>10</v>
       </c>
-      <c r="R39" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S39" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="T39" s="52" t="s">
+      <c r="R39" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S39" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="T39" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="U39" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="V39" s="52" t="s">
+      <c r="U39" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="V39" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="W39" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X39" s="56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="W39" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X39" s="50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="2:24" ht="15">
       <c r="B40" s="33"/>
       <c r="C40" s="33"/>
       <c r="D40" s="33"/>
@@ -2654,41 +2659,41 @@
       <c r="J40" s="33"/>
       <c r="K40" s="33"/>
       <c r="L40" s="33"/>
-      <c r="N40" s="53" t="s">
+      <c r="N40" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="52" t="s">
+      <c r="O40" s="46" t="s">
         <v>74</v>
       </c>
-      <c r="P40" s="52" t="s">
+      <c r="P40" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="Q40" s="52">
+      <c r="Q40" s="46">
         <v>10</v>
       </c>
-      <c r="R40" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="S40" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="T40" s="52" t="s">
+      <c r="R40" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="S40" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="T40" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="U40" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="V40" s="52" t="s">
+      <c r="U40" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="V40" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="W40" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="X40" s="56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="41" spans="2:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="W40" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="X40" s="50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="2:24" ht="15.75" thickBot="1">
       <c r="B41" s="33"/>
       <c r="C41" s="33"/>
       <c r="D41" s="33"/>
@@ -2700,41 +2705,41 @@
       <c r="J41" s="33"/>
       <c r="K41" s="33"/>
       <c r="L41" s="33"/>
-      <c r="N41" s="54" t="s">
+      <c r="N41" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="O41" s="55" t="s">
+      <c r="O41" s="49" t="s">
         <v>75</v>
       </c>
-      <c r="P41" s="55" t="s">
+      <c r="P41" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="Q41" s="55">
+      <c r="Q41" s="49">
         <v>10</v>
       </c>
-      <c r="R41" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="S41" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="T41" s="55" t="s">
+      <c r="R41" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="S41" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="T41" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="U41" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="V41" s="55" t="s">
+      <c r="U41" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="V41" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="W41" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="X41" s="57" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="42" spans="2:24" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="W41" s="49" t="s">
+        <v>15</v>
+      </c>
+      <c r="X41" s="51" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="2:24" ht="36" customHeight="1" thickBot="1">
       <c r="B42" s="33"/>
       <c r="C42" s="33"/>
       <c r="D42" s="33"/>
@@ -2747,7 +2752,7 @@
       <c r="K42" s="33"/>
       <c r="L42" s="33"/>
     </row>
-    <row r="43" spans="2:24" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:24" ht="18.75" thickBot="1">
       <c r="B43" s="33"/>
       <c r="C43" s="33"/>
       <c r="D43" s="33"/>
@@ -2759,21 +2764,21 @@
       <c r="J43" s="33"/>
       <c r="K43" s="33"/>
       <c r="L43" s="33"/>
-      <c r="N43" s="49" t="s">
+      <c r="N43" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="O43" s="50"/>
-      <c r="P43" s="50"/>
-      <c r="Q43" s="50"/>
-      <c r="R43" s="50"/>
-      <c r="S43" s="50"/>
-      <c r="T43" s="50"/>
-      <c r="U43" s="50"/>
-      <c r="V43" s="50"/>
-      <c r="W43" s="50"/>
-      <c r="X43" s="51"/>
-    </row>
-    <row r="44" spans="2:24" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O43" s="58"/>
+      <c r="P43" s="58"/>
+      <c r="Q43" s="58"/>
+      <c r="R43" s="58"/>
+      <c r="S43" s="58"/>
+      <c r="T43" s="58"/>
+      <c r="U43" s="58"/>
+      <c r="V43" s="58"/>
+      <c r="W43" s="58"/>
+      <c r="X43" s="59"/>
+    </row>
+    <row r="44" spans="2:24" ht="32.25" thickBot="1">
       <c r="B44" s="33"/>
       <c r="C44" s="33"/>
       <c r="D44" s="33"/>
@@ -2819,7 +2824,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:24">
       <c r="B45" s="33"/>
       <c r="C45" s="33"/>
       <c r="D45" s="33"/>
@@ -2865,7 +2870,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:24" ht="15" thickBot="1">
       <c r="B46" s="33"/>
       <c r="C46" s="33"/>
       <c r="D46" s="33"/>
@@ -2880,7 +2885,7 @@
       <c r="N46" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="O46" s="59" t="s">
+      <c r="O46" s="53" t="s">
         <v>81</v>
       </c>
       <c r="P46" s="11" t="s">
@@ -2911,7 +2916,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="2:24" ht="64.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:24" ht="64.900000000000006" customHeight="1" thickBot="1">
       <c r="B47" s="33"/>
       <c r="C47" s="33"/>
       <c r="D47" s="33"/>
@@ -2931,11 +2936,11 @@
       <c r="S47" s="28"/>
       <c r="T47" s="28"/>
       <c r="U47" s="28"/>
-      <c r="V47" s="58"/>
+      <c r="V47" s="52"/>
       <c r="W47" s="30"/>
-      <c r="X47" s="58"/>
-    </row>
-    <row r="48" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+      <c r="X47" s="52"/>
+    </row>
+    <row r="48" spans="2:24" ht="18">
       <c r="B48" s="33"/>
       <c r="C48" s="33"/>
       <c r="D48" s="33"/>
@@ -2947,21 +2952,21 @@
       <c r="J48" s="33"/>
       <c r="K48" s="33"/>
       <c r="L48" s="33"/>
-      <c r="N48" s="46" t="s">
+      <c r="N48" s="54" t="s">
         <v>82</v>
       </c>
-      <c r="O48" s="47"/>
-      <c r="P48" s="47"/>
-      <c r="Q48" s="47"/>
-      <c r="R48" s="47"/>
-      <c r="S48" s="47"/>
-      <c r="T48" s="47"/>
-      <c r="U48" s="47"/>
-      <c r="V48" s="47"/>
-      <c r="W48" s="47"/>
-      <c r="X48" s="48"/>
-    </row>
-    <row r="49" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O48" s="55"/>
+      <c r="P48" s="55"/>
+      <c r="Q48" s="55"/>
+      <c r="R48" s="55"/>
+      <c r="S48" s="55"/>
+      <c r="T48" s="55"/>
+      <c r="U48" s="55"/>
+      <c r="V48" s="55"/>
+      <c r="W48" s="55"/>
+      <c r="X48" s="56"/>
+    </row>
+    <row r="49" spans="2:24" ht="31.5">
       <c r="B49" s="33"/>
       <c r="C49" s="33"/>
       <c r="D49" s="33"/>
@@ -3007,7 +3012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:24">
       <c r="B50" s="33"/>
       <c r="C50" s="33"/>
       <c r="D50" s="33"/>
@@ -3053,7 +3058,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:24" ht="15" thickBot="1">
       <c r="B51" s="33"/>
       <c r="C51" s="33"/>
       <c r="D51" s="33"/>
@@ -3099,7 +3104,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:24">
       <c r="B52" s="33"/>
       <c r="C52" s="33"/>
       <c r="D52" s="33"/>
@@ -3119,11 +3124,11 @@
       <c r="S52" s="28"/>
       <c r="T52" s="28"/>
       <c r="U52" s="28"/>
-      <c r="V52" s="58"/>
+      <c r="V52" s="52"/>
       <c r="W52" s="30"/>
       <c r="X52" s="30"/>
     </row>
-    <row r="53" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:24">
       <c r="B53" s="33"/>
       <c r="C53" s="33"/>
       <c r="D53" s="33"/>
@@ -3143,11 +3148,11 @@
       <c r="S53" s="28"/>
       <c r="T53" s="28"/>
       <c r="U53" s="28"/>
-      <c r="V53" s="58"/>
+      <c r="V53" s="52"/>
       <c r="W53" s="30"/>
-      <c r="X53" s="58"/>
-    </row>
-    <row r="54" spans="2:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="X53" s="52"/>
+    </row>
+    <row r="54" spans="2:24" ht="22.15" customHeight="1">
       <c r="B54" s="33"/>
       <c r="C54" s="33"/>
       <c r="D54" s="33"/>
@@ -3169,9 +3174,9 @@
       <c r="U54" s="28"/>
       <c r="V54" s="30"/>
       <c r="W54" s="30"/>
-      <c r="X54" s="58"/>
-    </row>
-    <row r="55" spans="2:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="X54" s="52"/>
+    </row>
+    <row r="55" spans="2:24" ht="36" customHeight="1">
       <c r="B55" s="33"/>
       <c r="C55" s="33"/>
       <c r="D55" s="33"/>
@@ -3195,7 +3200,7 @@
       <c r="W55" s="30"/>
       <c r="X55" s="28"/>
     </row>
-    <row r="56" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:24" ht="42" customHeight="1">
       <c r="B56" s="33"/>
       <c r="C56" s="33"/>
       <c r="D56" s="33"/>
@@ -3208,7 +3213,7 @@
       <c r="K56" s="33"/>
       <c r="L56" s="33"/>
     </row>
-    <row r="57" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:24" ht="42" customHeight="1">
       <c r="B57" s="33"/>
       <c r="C57" s="33"/>
       <c r="D57" s="33"/>
@@ -3221,7 +3226,7 @@
       <c r="K57" s="33"/>
       <c r="L57" s="33"/>
     </row>
-    <row r="58" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:24" ht="42" customHeight="1">
       <c r="B58" s="33"/>
       <c r="C58" s="33"/>
       <c r="D58" s="33"/>
@@ -3234,7 +3239,7 @@
       <c r="K58" s="33"/>
       <c r="L58" s="33"/>
     </row>
-    <row r="59" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:24" ht="42" customHeight="1">
       <c r="B59" s="33"/>
       <c r="C59" s="33"/>
       <c r="D59" s="33"/>
@@ -3247,7 +3252,7 @@
       <c r="K59" s="33"/>
       <c r="L59" s="33"/>
     </row>
-    <row r="60" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:24" ht="42" customHeight="1">
       <c r="B60" s="33"/>
       <c r="C60" s="33"/>
       <c r="D60" s="33"/>
@@ -3260,7 +3265,7 @@
       <c r="K60" s="33"/>
       <c r="L60" s="33"/>
     </row>
-    <row r="61" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:24" ht="42" customHeight="1">
       <c r="B61" s="33"/>
       <c r="C61" s="33"/>
       <c r="D61" s="33"/>
@@ -3274,7 +3279,7 @@
       <c r="L61" s="33"/>
       <c r="M61" s="19"/>
     </row>
-    <row r="62" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:24" ht="42" customHeight="1">
       <c r="B62" s="33"/>
       <c r="C62" s="33"/>
       <c r="D62" s="33"/>
@@ -3287,7 +3292,7 @@
       <c r="K62" s="33"/>
       <c r="L62" s="33"/>
     </row>
-    <row r="63" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:24" ht="42" customHeight="1">
       <c r="B63" s="33"/>
       <c r="C63" s="33"/>
       <c r="D63" s="33"/>

</xml_diff>